<commit_message>
try to fix later
</commit_message>
<xml_diff>
--- a/Backend/productos_sin_stock.xlsx
+++ b/Backend/productos_sin_stock.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -524,6 +524,18 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>R933979</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-07-13 16:14:14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
update to implement actually
</commit_message>
<xml_diff>
--- a/Backend/productos_sin_stock.xlsx
+++ b/Backend/productos_sin_stock.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,10 +424,15 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Descripción</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Stock Fantasma</t>
         </is>
@@ -441,10 +446,15 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>FILTRO PAÑO LAVABLE  X MT2   RE</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>2026-07-13 10:12:23</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>0.42</v>
       </c>
     </row>
@@ -456,10 +466,15 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>Termost.RANCO K59L1132  ARB420 27053 hel</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>2026-07-13 10:12:35</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -471,10 +486,15 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>Termost.RANCO K59L2698 1.05 MTS SE REEMPLA R816606</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>2026-07-13 10:13:23</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>2</v>
       </c>
     </row>
@@ -486,10 +506,15 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-13 10:15:34</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
+          <t>TERMOST. B S  RC94526-2S PATRICK EL FRIO NO SE VA!</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TERMOST. B S  RC94526-2S PATRICK EL FRIO NO SE VA!</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -501,10 +526,15 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>TAPA FUGAS ACH ANTON JERINGA X6ML</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>2026-07-13 11:53:17</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>13</v>
       </c>
     </row>
@@ -516,10 +546,15 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-13 12:32:57</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
+          <t>SEP. ACEITE "BLUE STAR"XFB5303 7/8 DESARMABLE</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SEP. ACEITE "BLUE STAR"XFB5303 7/8 DESARMABLE</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -531,10 +566,15 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-13 12:38:30</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
+          <t>Tubo recibidor"BlueStar"XF-1.0L---- 1lt-</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Tubo recibidor"BlueStar"XF-1.0L---- 1lt-</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -546,10 +586,15 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-13 14:31:35</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
+          <t>FUNDENTE BLUESTAR FLUX-115gr.-</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>FUNDENTE BLUESTAR FLUX-115gr.-</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
         <v>1</v>
       </c>
     </row>
@@ -561,10 +606,15 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>FORZADOR 13 VOLTS 3,3 WHATS</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>2026-07-13 16:14:14</t>
         </is>
       </c>
-      <c r="C10" t="n">
+      <c r="D10" t="n">
         <v>1</v>
       </c>
     </row>
@@ -576,11 +626,36 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>PALA U. COND. DIAM. 40CM 3 ASPAS BUJE 8MM IZQ.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>2026-07-13 16:36:37</t>
         </is>
       </c>
-      <c r="C11" t="n">
+      <c r="D11" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>R920759</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>LATA GENERICO YH-12 PLUSS 680 GR</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>LATA GENERICO YH-12 PLUSS 680 GR</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: change app desktop
</commit_message>
<xml_diff>
--- a/Backend/productos_sin_stock.xlsx
+++ b/Backend/productos_sin_stock.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -741,6 +741,66 @@
         <v>1</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>R131530</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>AISLACION DE PVC 3M TAPA TRASERA WRM40D</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-07-16 14:58:38</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>R911041</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>MENSULA M-1270</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MENSULA M-1270</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>R139650</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>PALAS DI-CALL 5 ASPAS Ø 300 C/ BUJE 9.5 MM</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>PALAS DI-CALL 5 ASPAS Ø 300 C/ BUJE 9.5 MM</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>